<commit_message>
Update comparison data file to correct SE
</commit_message>
<xml_diff>
--- a/ExplicitSimulations/Data/ComparisonData.xlsx
+++ b/ExplicitSimulations/Data/ComparisonData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2130652544840/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2141903994903/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{7106D4D6-35E8-4BBD-AC7A-416BA6142B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{963DB047-7D59-446C-A179-17B6C089AF8A}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="8_{7106D4D6-35E8-4BBD-AC7A-416BA6142B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEA7FFCF-867E-49B9-9F17-A254E09D58E4}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{13A0BBB6-7A72-4064-9F4D-BE11A7F05FD0}"/>
+    <workbookView xWindow="38280" yWindow="5175" windowWidth="29040" windowHeight="15720" xr2:uid="{13A0BBB6-7A72-4064-9F4D-BE11A7F05FD0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -429,9 +429,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{565550E5-04CF-44D6-9392-7D38F9F0B00E}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -454,7 +454,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -462,10 +462,10 @@
         <v>0.23</v>
       </c>
       <c r="C2">
-        <v>0.16200000000000001</v>
+        <v>0.16800000000000001</v>
       </c>
       <c r="D2">
-        <v>0.29699999999999999</v>
+        <v>0.28899999999999998</v>
       </c>
       <c r="E2">
         <v>0.05</v>
@@ -477,7 +477,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -485,10 +485,10 @@
         <v>0.31</v>
       </c>
       <c r="C3">
-        <v>0.26100000000000001</v>
+        <v>0.26500000000000001</v>
       </c>
       <c r="D3">
-        <v>0.35699999999999998</v>
+        <v>0.35099999999999998</v>
       </c>
       <c r="E3">
         <v>0.16</v>
@@ -500,7 +500,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -508,10 +508,10 @@
         <v>0.39</v>
       </c>
       <c r="C4">
-        <v>0.307</v>
+        <v>0.316</v>
       </c>
       <c r="D4">
-        <v>0.47599999999999998</v>
+        <v>0.46700000000000003</v>
       </c>
       <c r="E4">
         <v>0.27</v>
@@ -523,7 +523,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -531,10 +531,10 @@
         <v>0.47</v>
       </c>
       <c r="C5">
-        <v>0.4</v>
+        <v>0.40699999999999997</v>
       </c>
       <c r="D5">
-        <v>0.54200000000000004</v>
+        <v>0.53400000000000003</v>
       </c>
       <c r="E5">
         <v>0.38</v>
@@ -546,7 +546,7 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -554,10 +554,10 @@
         <v>0.6</v>
       </c>
       <c r="C6">
-        <v>0.504</v>
+        <v>0.51300000000000001</v>
       </c>
       <c r="D6">
-        <v>0.68799999999999994</v>
+        <v>0.67800000000000005</v>
       </c>
       <c r="E6">
         <v>0.47</v>
@@ -569,7 +569,7 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>

</xml_diff>